<commit_message>
improvement: added functionality for passing URLs dynamically using command line arguement
</commit_message>
<xml_diff>
--- a/my_crawler_project/visited_links.xlsx
+++ b/my_crawler_project/visited_links.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A25"/>
+  <dimension ref="A1:A2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -438,168 +438,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>https://thestjgroup.com/mohali-citi-centre-walk</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>https://thestjgroup.com/#hero</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>https://thestjgroup.com/mohali-citi-centre-3</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>https://thestjgroup.com/the-pinnacle</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>https://thestjgroup.com/#section-2</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>https://thestjgroup.com/about</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>https://thestjgroup.com/mohali-citi-centre-avenue</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>https://thestjgroup.com/sunaar-the-jeweller</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>https://thestjgroup.com/residential</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>https://thestjgroup.com/mohali-citi-centre-4</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>https://thestjgroup.com/the-bazaar</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>https://thestjgroup.com/mohali-citi-centre-2</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>https://thestjgroup.com/mohali-citi-centre-1</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>https://thestjgroup.com/saraf-the-jeweller#hero</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>https://thestjgroup.com/whatsapp-communication-opt-in-policy</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>https://thestjgroup.com/mohali-citi-centre-square</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>https://thestjgroup.com/mohali-citi-centre-1#section-2</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>https://thestjgroup.com/industrial</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>https://thestjgroup.com/saraf-the-jeweller</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>https://thestjgroup.com/commercial</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>https://thestjgroup.com/projects</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>https://thestjgroup.com/contact</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>https://thestjgroup.com/our-ventures</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>https://thestjgroup.com/</t>
+          <t>https://thestjgroup.com</t>
         </is>
       </c>
     </row>

</xml_diff>